<commit_message>
081925 - updated week 2 bad external link
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 16.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 16.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
-  <workbookPr/>
+  <workbookPr updateLinks="always"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204337AF-8863-DD46-AF0E-BF0A4C2C9D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3181B8A7-654A-CA4E-BB38-B19FF68D8EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1300" yWindow="500" windowWidth="28100" windowHeight="19840" firstSheet="3" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1300" yWindow="500" windowWidth="28100" windowHeight="19840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="14" r:id="rId1"/>
@@ -402,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -545,28 +545,9 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -605,6 +586,22 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1080,23 +1077,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1110,25 +1107,25 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="60"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
       <c r="T2" s="29"/>
@@ -1155,8 +1152,8 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="5"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="29"/>
@@ -1168,7 +1165,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="55" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -1213,8 +1210,8 @@
       <c r="O4" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="P4" s="61"/>
-      <c r="Q4" s="62"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="27"/>
       <c r="S4" s="3"/>
       <c r="T4" s="30"/>
@@ -1226,7 +1223,7 @@
       <c r="Z4" s="3"/>
     </row>
     <row r="5" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A5" s="65"/>
+      <c r="A5" s="56"/>
       <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
@@ -1264,8 +1261,8 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="22"/>
-      <c r="P5" s="61"/>
-      <c r="Q5" s="63"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="32"/>
       <c r="R5" s="4"/>
       <c r="S5" s="3"/>
       <c r="T5" s="30"/>
@@ -1277,7 +1274,7 @@
       <c r="Z5" s="3"/>
     </row>
     <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="66"/>
+      <c r="A6" s="57"/>
       <c r="B6" s="24" t="s">
         <v>24</v>
       </c>
@@ -1325,7 +1322,7 @@
       <c r="Z6" s="3"/>
     </row>
     <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A7" s="67"/>
+      <c r="A7" s="58"/>
       <c r="B7" s="12" t="s">
         <v>23</v>
       </c>
@@ -1361,7 +1358,7 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="68"/>
+      <c r="A8" s="59"/>
       <c r="B8" s="16" t="s">
         <v>25</v>
       </c>
@@ -1423,7 +1420,7 @@
       <c r="Z8" s="33"/>
     </row>
     <row r="9" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A9" s="67"/>
+      <c r="A9" s="58"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -1450,7 +1447,7 @@
       <c r="T9" s="2"/>
     </row>
     <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="68"/>
+      <c r="A10" s="59"/>
       <c r="B10" s="16"/>
       <c r="C10" s="16" t="str">
         <f>IF(C9&gt;0, VLOOKUP(C9-C$5-(INT($M9/9)+(MOD($M9,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1504,7 +1501,7 @@
       <c r="T10" s="2"/>
     </row>
     <row r="11" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A11" s="67"/>
+      <c r="A11" s="58"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -1532,7 +1529,7 @@
       <c r="T11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="68"/>
+      <c r="A12" s="59"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16" t="str">
         <f>IF(C11&gt;0, VLOOKUP(C11-C$5-(INT($M11/9)+(MOD($M11,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1587,7 +1584,7 @@
       <c r="T12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A13" s="67"/>
+      <c r="A13" s="58"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -1615,7 +1612,7 @@
       <c r="T13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="68"/>
+      <c r="A14" s="59"/>
       <c r="B14" s="16"/>
       <c r="C14" s="16" t="str">
         <f>IF(C13&gt;0, VLOOKUP(C13-C$5-(INT($M13/9)+(MOD($M13,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1670,7 +1667,7 @@
       <c r="T14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A15" s="67"/>
+      <c r="A15" s="58"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -1701,7 +1698,7 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="68"/>
+      <c r="A16" s="59"/>
       <c r="B16" s="16"/>
       <c r="C16" s="16" t="str">
         <f>IF(C15&gt;0, VLOOKUP(C15-C$5-(INT($M15/9)+(MOD($M15,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1759,7 +1756,7 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A17" s="67"/>
+      <c r="A17" s="58"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -1790,7 +1787,7 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="68"/>
+      <c r="A18" s="59"/>
       <c r="B18" s="16"/>
       <c r="C18" s="16" t="str">
         <f>IF(C17&gt;0, VLOOKUP(C17-C$5-(INT($M17/9)+(MOD($M17,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1848,7 +1845,7 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A19" s="67"/>
+      <c r="A19" s="58"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -1875,7 +1872,7 @@
       <c r="T19" s="2"/>
     </row>
     <row r="20" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="68"/>
+      <c r="A20" s="59"/>
       <c r="B20" s="16"/>
       <c r="C20" s="16" t="str">
         <f>IF(C19&gt;0, VLOOKUP(C19-C$5-(INT($M19/9)+(MOD($M19,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -1968,23 +1965,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1998,23 +1995,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -2056,7 +2053,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -3536,23 +3533,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -3566,23 +3563,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -3624,7 +3621,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -4867,23 +4864,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -4897,23 +4894,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -4955,7 +4952,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -6318,23 +6315,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -6348,23 +6345,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -6406,7 +6403,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -8120,23 +8117,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -8150,23 +8147,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -8208,7 +8205,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -9922,23 +9919,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -9952,23 +9949,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -10010,7 +10007,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -11724,23 +11721,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -11754,23 +11751,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -11812,7 +11809,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -13476,23 +13473,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -13506,23 +13503,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -13564,7 +13561,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -15278,23 +15275,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -15308,23 +15305,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -15366,7 +15363,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -18079,23 +18076,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -18109,23 +18106,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -18167,7 +18164,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -19029,23 +19026,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -19059,23 +19056,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -19117,7 +19114,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -19337,39 +19334,39 @@
         <v>25</v>
       </c>
       <c r="C8" s="16">
-        <f>IF(C7&gt;0, VLOOKUP(C7-C$5-(INT($M7/9)+(MOD($M7,9)&gt;=C$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(C7&gt;0, VLOOKUP(C7-C$5-(INT($M7/9)+(MOD($M7,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
       <c r="D8" s="16">
-        <f>IF(D7&gt;0, VLOOKUP(D7-D$5-(INT($M7/9)+(MOD($M7,9)&gt;=D$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(D7&gt;0, VLOOKUP(D7-D$5-(INT($M7/9)+(MOD($M7,9)&gt;=D$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="16">
-        <f>IF(E7&gt;0, VLOOKUP(E7-E$5-(INT($M7/9)+(MOD($M7,9)&gt;=E$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(E7&gt;0, VLOOKUP(E7-E$5-(INT($M7/9)+(MOD($M7,9)&gt;=E$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>4</v>
       </c>
       <c r="F8" s="16">
-        <f>IF(F7&gt;0, VLOOKUP(F7-F$5-(INT($M7/9)+(MOD($M7,9)&gt;=F$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(F7&gt;0, VLOOKUP(F7-F$5-(INT($M7/9)+(MOD($M7,9)&gt;=F$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
       <c r="G8" s="16">
-        <f>IF(G7&gt;0, VLOOKUP(G7-G$5-(INT($M7/9)+(MOD($M7,9)&gt;=G$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(G7&gt;0, VLOOKUP(G7-G$5-(INT($M7/9)+(MOD($M7,9)&gt;=G$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
       <c r="H8" s="16">
-        <f>IF(H7&gt;0, VLOOKUP(H7-H$5-(INT($M7/9)+(MOD($M7,9)&gt;=H$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(H7&gt;0, VLOOKUP(H7-H$5-(INT($M7/9)+(MOD($M7,9)&gt;=H$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
       <c r="I8" s="16">
-        <f>IF(I7&gt;0, VLOOKUP(I7-I$5-(INT($M7/9)+(MOD($M7,9)&gt;=I$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(I7&gt;0, VLOOKUP(I7-I$5-(INT($M7/9)+(MOD($M7,9)&gt;=I$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
       <c r="J8" s="16">
-        <f>IF(J7&gt;0, VLOOKUP(J7-J$5-(INT($M7/9)+(MOD($M7,9)&gt;=J$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(J7&gt;0, VLOOKUP(J7-J$5-(INT($M7/9)+(MOD($M7,9)&gt;=J$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
       <c r="K8" s="16">
-        <f>IF(K7&gt;0, VLOOKUP(K7-K$5-(INT($M7/9)+(MOD($M7,9)&gt;=K$6)), '[1]Point System'!$A$4:$B$15, 2),"")</f>
+        <f>IF(K7&gt;0, VLOOKUP(K7-K$5-(INT($M7/9)+(MOD($M7,9)&gt;=K$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
       <c r="L8" s="17">
@@ -20711,23 +20708,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -20741,23 +20738,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -20799,7 +20796,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -21649,7 +21646,7 @@
   <dimension ref="A1:Z10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="73" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" style="64" customWidth="1"/>
     <col min="2" max="2" width="9.1640625" style="34" bestFit="1" customWidth="1"/>
     <col min="3" max="11" width="5" style="34" customWidth="1"/>
     <col min="12" max="12" width="5.1640625" style="34" bestFit="1" customWidth="1"/>
@@ -21661,23 +21658,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="17" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
+      <c r="A1" s="71" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
       <c r="P1" s="35"/>
       <c r="Q1" s="35"/>
       <c r="R1" s="35"/>
@@ -21691,23 +21688,23 @@
       <c r="Z1" s="35"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
+      <c r="A2" s="73" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
       <c r="P2" s="35"/>
       <c r="Q2" s="35"/>
       <c r="R2" s="35"/>
@@ -21721,7 +21718,7 @@
       <c r="Z2" s="35"/>
     </row>
     <row r="3" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="69"/>
+      <c r="A3" s="60"/>
       <c r="B3" s="35"/>
       <c r="C3" s="37"/>
       <c r="D3" s="37"/>
@@ -21749,7 +21746,7 @@
       <c r="Z3" s="35"/>
     </row>
     <row r="4" spans="1:26" ht="40" x14ac:dyDescent="0.2">
-      <c r="A4" s="70" t="s">
+      <c r="A4" s="61" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="39" t="s">
@@ -21807,7 +21804,7 @@
       <c r="Z4" s="36"/>
     </row>
     <row r="5" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A5" s="71"/>
+      <c r="A5" s="62"/>
       <c r="B5" s="41" t="s">
         <v>10</v>
       </c>
@@ -21858,7 +21855,7 @@
       <c r="Z5" s="36"/>
     </row>
     <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="72"/>
+      <c r="A6" s="63"/>
       <c r="B6" s="44" t="s">
         <v>24</v>
       </c>
@@ -21906,7 +21903,7 @@
       <c r="Z6" s="36"/>
     </row>
     <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A7" s="74" t="s">
+      <c r="A7" s="65" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="47" t="s">
@@ -21964,7 +21961,7 @@
       <c r="Z7" s="35"/>
     </row>
     <row r="8" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="75"/>
+      <c r="A8" s="66"/>
       <c r="B8" s="50" t="s">
         <v>25</v>
       </c>
@@ -22027,7 +22024,7 @@
       <c r="Z8" s="35"/>
     </row>
     <row r="9" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="65" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="47"/>
@@ -22083,7 +22080,7 @@
       <c r="Z9" s="35"/>
     </row>
     <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="75"/>
+      <c r="A10" s="66"/>
       <c r="B10" s="50"/>
       <c r="C10" s="16">
         <f>IF(C9&gt;0, VLOOKUP(C9-C$5-(INT($M9/9)+(MOD($M9,9)&gt;=C$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
@@ -22173,23 +22170,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -22203,23 +22200,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -22261,7 +22258,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -23237,23 +23234,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -23267,23 +23264,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -23325,7 +23322,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
@@ -24793,23 +24790,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
+      <c r="A1" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -24823,23 +24820,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
+      <c r="A2" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -24881,7 +24878,7 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="19" t="s">

</xml_diff>

<commit_message>
081925 - updated week 16 skins
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 16.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3181B8A7-654A-CA4E-BB38-B19FF68D8EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A66946-756E-684D-B434-9E4DCC9E386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1300" yWindow="500" windowWidth="28100" windowHeight="19840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1300" yWindow="500" windowWidth="14320" windowHeight="19840" firstSheet="11" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="14" r:id="rId1"/>

</xml_diff>